<commit_message>
implemented spatial demography parsing
- raster files with layers containing scaling factors for demographic rates (max. stages*sexes*3) for each landscape
- table for assigning layer number to each stages/sex for the 3 different demographic rates

is compiling, but need to run tests
</commit_message>
<xml_diff>
--- a/doc/Manual/Batchmode/LandFile.xlsx
+++ b/doc/Manual/Batchmode/LandFile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\s02tp3\github\rs_batch_dev\doc\Manual\Batchmode\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jreeg.IBB\RangeShiftR\transloc_new_genetics_spatial_demog\RangeShifter_batch\doc\Manual\Batchmode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34BDD6A0-11A8-435D-91BF-E87C9D2405AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AB82FA-11CD-4C15-B2DF-5E11E88F3AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description - imported" sheetId="3" r:id="rId1"/>
@@ -19,15 +19,21 @@
     <sheet name="Imported cell-based 1" sheetId="9" r:id="rId4"/>
     <sheet name="Imported cell-based 2" sheetId="8" r:id="rId5"/>
     <sheet name="Description - Dynamic Land File" sheetId="10" r:id="rId6"/>
-    <sheet name="Description - artificial" sheetId="6" r:id="rId7"/>
-    <sheet name="Artificial" sheetId="5" r:id="rId8"/>
+    <sheet name="Description - Spatial demograph" sheetId="11" r:id="rId7"/>
+    <sheet name="Description - artificial" sheetId="6" r:id="rId8"/>
+    <sheet name="Artificial" sheetId="5" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -35,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="83">
   <si>
     <t>Fractal</t>
   </si>
@@ -251,6 +257,39 @@
   </si>
   <si>
     <t>Dimension (number of cells) along the y axis</t>
+  </si>
+  <si>
+    <t>SpatialDemogFile</t>
+  </si>
+  <si>
+    <t>Required only if spatially varying demographic rates are simulated, otherwise NULL</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>spatialdemog001.txt</t>
+  </si>
+  <si>
+    <t>Filename</t>
+  </si>
+  <si>
+    <t>Name of the map holding the factors applied to the standard demographic rates.</t>
+  </si>
+  <si>
+    <t>Must be sequential numbers starting with 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This number is referred to when you assign a layer to a demographic rate. </t>
+  </si>
+  <si>
+    <t>Must match the extension of the habitat map</t>
+  </si>
+  <si>
+    <t>Name of the file containing the information on spatial demographic rates (*.txt)</t>
+  </si>
+  <si>
+    <t>NbOfLayer</t>
   </si>
 </sst>
 </file>
@@ -641,7 +680,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -797,6 +836,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -846,7 +896,7 @@
     <xf numFmtId="0" fontId="27" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -895,6 +945,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="41" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="41" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="34" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="46">
     <cellStyle name="20% - Accent1" xfId="18" builtinId="30" customBuiltin="1"/>
@@ -1244,16 +1304,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="57.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="72.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>24</v>
       </c>
@@ -1267,7 +1327,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -1281,7 +1341,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>15</v>
       </c>
@@ -1295,7 +1355,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
@@ -1309,7 +1369,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>16</v>
       </c>
@@ -1323,7 +1383,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
         <v>62</v>
       </c>
@@ -1337,31 +1397,45 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="33" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B8" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C8" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D8" s="24" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+    <row r="9" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B9" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C9" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D9" s="13" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1373,19 +1447,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.88671875" customWidth="1"/>
+    <col min="5" max="5" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.90625" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>12</v>
       </c>
@@ -1407,8 +1481,11 @@
       <c r="G1" s="10" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="12">
         <v>21</v>
       </c>
@@ -1430,8 +1507,11 @@
       <c r="G2" s="21" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="12">
         <v>22</v>
       </c>
@@ -1453,8 +1533,11 @@
       <c r="G3" s="21" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="12">
         <v>23</v>
       </c>
@@ -1476,8 +1559,11 @@
       <c r="G4" s="21" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="12">
         <v>24</v>
       </c>
@@ -1499,8 +1585,11 @@
       <c r="G5" s="16" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="12">
         <v>25</v>
       </c>
@@ -1521,6 +1610,35 @@
       </c>
       <c r="G6" s="16" t="s">
         <v>36</v>
+      </c>
+      <c r="H6" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="31">
+        <v>26</v>
+      </c>
+      <c r="B7" s="31">
+        <v>2</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" s="32" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1532,18 +1650,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>12</v>
       </c>
@@ -1566,7 +1684,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="12">
         <v>21</v>
       </c>
@@ -1589,7 +1707,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="12">
         <v>22</v>
       </c>
@@ -1621,18 +1739,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.08984375" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>12</v>
       </c>
@@ -1655,7 +1773,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="12">
         <v>21</v>
       </c>
@@ -1678,7 +1796,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="12">
         <v>22</v>
       </c>
@@ -1701,7 +1819,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="12">
         <v>23</v>
       </c>
@@ -1724,7 +1842,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="12">
         <v>24</v>
       </c>
@@ -1747,7 +1865,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="12">
         <v>25</v>
       </c>
@@ -1779,18 +1897,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>12</v>
       </c>
@@ -1813,7 +1931,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="12">
         <v>21</v>
       </c>
@@ -1836,7 +1954,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="12">
         <v>22</v>
       </c>
@@ -1867,16 +1985,16 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="4" width="57.5546875" customWidth="1"/>
+    <col min="4" max="4" width="57.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>24</v>
       </c>
@@ -1890,7 +2008,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>54</v>
       </c>
@@ -1904,7 +2022,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>55</v>
       </c>
@@ -1918,7 +2036,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>56</v>
       </c>
@@ -1932,7 +2050,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>57</v>
       </c>
@@ -1946,7 +2064,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="22" t="s">
         <v>67</v>
       </c>
@@ -1958,6 +2076,20 @@
       </c>
       <c r="D6" s="24" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1967,17 +2099,74 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26ABD0B5-63B0-47F0-AB66-A126FB67DC78}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="63.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="47.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="63.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>24</v>
       </c>
@@ -1991,7 +2180,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -2005,7 +2194,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>0</v>
       </c>
@@ -2017,7 +2206,7 @@
       </c>
       <c r="D3" s="14"/>
     </row>
-    <row r="4" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>2</v>
       </c>
@@ -2029,7 +2218,7 @@
       </c>
       <c r="D4" s="14"/>
     </row>
-    <row r="5" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
@@ -2043,7 +2232,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
@@ -2055,7 +2244,7 @@
       </c>
       <c r="D6" s="29"/>
     </row>
-    <row r="7" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
@@ -2069,7 +2258,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -2083,7 +2272,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>37</v>
       </c>
@@ -2095,7 +2284,7 @@
       </c>
       <c r="D9" s="14"/>
     </row>
-    <row r="10" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
@@ -2118,12 +2307,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:9" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
         <v>12</v>
       </c>
@@ -2152,7 +2341,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -2181,7 +2370,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -2210,7 +2399,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -2239,7 +2428,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="17">
         <v>4</v>
       </c>

</xml_diff>